<commit_message>
Add new feature - delete-empty-rows
</commit_message>
<xml_diff>
--- a/tests/fixtures/preserved_artifacts.xlsx
+++ b/tests/fixtures/preserved_artifacts.xlsx
@@ -5,18 +5,31 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\wsl\project\excel-fillna\tests\fixtures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\wsl\project\excel-fill-na\tests\fixtures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{828D28A7-FB58-42FC-96E9-361320B84AC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E32B0ED-148D-4748-80E6-A7928E221618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
     <sheet name="Other" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -26,7 +39,7 @@
     <author>tc={A8F2A416-1695-4403-851D-20179B92388B}</author>
   </authors>
   <commentList>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{A8F2A416-1695-4403-851D-20179B92388B}">
+    <comment ref="D6" authorId="0" shapeId="0" xr:uid="{A8F2A416-1695-4403-851D-20179B92388B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -62,9 +75,6 @@
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>header</t>
-  </si>
   <si>
     <t>chart anchor</t>
   </si>
@@ -86,12 +96,15 @@
   <si>
     <t>20250521 Draft [Annex 1] Trend Chart Panel</t>
   </si>
+  <si>
+    <t>a</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,12 +119,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -140,10 +147,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -370,16 +381,16 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>317500</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>82550</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>29210</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>82550</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>142240</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>8890</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -408,8 +419,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="317500" y="1187450"/>
-          <a:ext cx="2578100" cy="2578100"/>
+          <a:off x="638810" y="2194560"/>
+          <a:ext cx="2555240" cy="2565400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -776,7 +787,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="D5" dT="2026-04-06T16:12:55.54" personId="{C0AF02FF-D953-497C-8EDA-E4968AC9B1B3}" id="{A8F2A416-1695-4403-851D-20179B92388B}">
+  <threadedComment ref="D6" dT="2026-04-06T16:12:55.54" personId="{C0AF02FF-D953-497C-8EDA-E4968AC9B1B3}" id="{A8F2A416-1695-4403-851D-20179B92388B}">
     <text>asdad</text>
   </threadedComment>
 </ThreadedComments>
@@ -784,55 +795,76 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
       <c r="C1" s="1"/>
+      <c r="E1" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="F1">
         <v>1</v>
       </c>
       <c r="H1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E2" s="3"/>
       <c r="F2">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
+      <c r="E3" s="3"/>
       <c r="F3">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35"/>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A5" s="3"/>
+      <c r="D5" s="2"/>
+    </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="D6" t="s">
-        <v>4</v>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B7" s="4"/>
+      <c r="D7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="F10" t="str">
+        <f>E1</f>
+        <v>a</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="E1:E3"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A5:A6"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" xr:uid="{335E8BA8-7803-460F-A1C5-17E4726CF3C1}"/>
   </hyperlinks>
@@ -849,12 +881,12 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>